<commit_message>
auto: snapshot 2026-08-02 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3223.xlsx
+++ b/clan_3223.xlsx
@@ -9235,7 +9235,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-02 13:01:00</t>
+          <t>Timestamp: 2026-08-02 13:31:00</t>
         </is>
       </c>
     </row>
@@ -9758,11 +9758,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>1650</v>
+        <v>1710</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+617</t>
+          <t>+677</t>
         </is>
       </c>
     </row>
@@ -9803,11 +9803,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>5822</v>
+        <v>6062</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+1061</t>
+          <t>+1301</t>
         </is>
       </c>
     </row>
@@ -9983,11 +9983,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>24624</v>
+        <v>24664</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+1592</t>
+          <t>+1632</t>
         </is>
       </c>
     </row>
@@ -9998,11 +9998,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>6269</v>
+        <v>6329</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+2024</t>
+          <t>+2084</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-03 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3223.xlsx
+++ b/clan_3223.xlsx
@@ -10979,7 +10979,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-03 13:01:00</t>
+          <t>Timestamp: 2026-08-03 13:31:00</t>
         </is>
       </c>
     </row>
@@ -11322,11 +11322,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>18102</v>
+        <v>18132</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+2319</t>
+          <t>+2349</t>
         </is>
       </c>
     </row>
@@ -11472,11 +11472,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>20130</v>
+        <v>20160</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1230</t>
         </is>
       </c>
     </row>
@@ -11727,11 +11727,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>27097</v>
+        <v>27127</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+2433</t>
+          <t>+2463</t>
         </is>
       </c>
     </row>
@@ -11787,11 +11787,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>23726</v>
+        <v>23756</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+1644</t>
+          <t>+1674</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-06 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3223.xlsx
+++ b/clan_3223.xlsx
@@ -13619,7 +13619,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-06 13:01:00</t>
+          <t>Timestamp: 2026-08-06 13:31:00</t>
         </is>
       </c>
     </row>
@@ -14217,11 +14217,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>27043</v>
+        <v>27103</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+2170</t>
+          <t>+2230</t>
         </is>
       </c>
     </row>
@@ -14232,11 +14232,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>37155</v>
+        <v>37215</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+2776</t>
+          <t>+2836</t>
         </is>
       </c>
     </row>
@@ -14247,11 +14247,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>26602</v>
+        <v>26662</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+2170</t>
+          <t>+2230</t>
         </is>
       </c>
     </row>
@@ -14262,11 +14262,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>2380</v>
+        <v>2440</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+1220</t>
+          <t>+1280</t>
         </is>
       </c>
     </row>
@@ -14277,11 +14277,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>36326</v>
+        <v>36386</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+2469</t>
+          <t>+2529</t>
         </is>
       </c>
     </row>
@@ -14367,11 +14367,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>30788</v>
+        <v>30848</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+2191</t>
+          <t>+2251</t>
         </is>
       </c>
     </row>
@@ -14427,11 +14427,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>26744</v>
+        <v>26804</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+1980</t>
+          <t>+2040</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-10 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3223.xlsx
+++ b/clan_3223.xlsx
@@ -17139,7 +17139,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-10 13:01:00</t>
+          <t>Timestamp: 2026-08-10 13:31:00</t>
         </is>
       </c>
     </row>
@@ -17767,11 +17767,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>1128</v>
+        <v>1278</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>-63571</t>
+          <t>-63421</t>
         </is>
       </c>
     </row>
@@ -17872,11 +17872,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>719</v>
+        <v>797</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>-54588</t>
+          <t>-54510</t>
         </is>
       </c>
     </row>
@@ -17887,11 +17887,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>1073</v>
+        <v>1223</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>-38851</t>
+          <t>-38701</t>
         </is>
       </c>
     </row>
@@ -17902,11 +17902,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>848</v>
+        <v>998</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>-24316</t>
+          <t>-24166</t>
         </is>
       </c>
     </row>
@@ -17932,11 +17932,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>918</v>
+        <v>924</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>-49548</t>
+          <t>-49542</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-12 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3223.xlsx
+++ b/clan_3223.xlsx
@@ -18869,7 +18869,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-12 13:01:00</t>
+          <t>Timestamp: 2026-08-12 13:31:00</t>
         </is>
       </c>
     </row>
@@ -19422,11 +19422,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>4438</v>
+        <v>4498</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+2486</t>
+          <t>+2546</t>
         </is>
       </c>
     </row>
@@ -19467,11 +19467,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>8191</v>
+        <v>8251</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+3109</t>
+          <t>+3169</t>
         </is>
       </c>
     </row>
@@ -19557,11 +19557,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>5629</v>
+        <v>5689</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+3283</t>
+          <t>+3343</t>
         </is>
       </c>
     </row>
@@ -19617,11 +19617,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>5603</v>
+        <v>5663</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+3266</t>
+          <t>+3326</t>
         </is>
       </c>
     </row>
@@ -19647,11 +19647,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>5742</v>
+        <v>5802</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+2627</t>
+          <t>+2687</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-14 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3223.xlsx
+++ b/clan_3223.xlsx
@@ -36,6 +36,7 @@
     <sheet name="2026-08-10" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="2026-08-11" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="2026-08-12" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="2026-08-14" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20543,6 +20544,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sigma Brothers (3223)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-14 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>MAHORAGA</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>WoKy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>128</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>H U N T E R</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>SB ELISEUS</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>INFERNO</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>6493</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+1922</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Hydra anbu™</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Kyara Senju™</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>1105</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+1105</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Toka Senju™</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>GOJU</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>The prince JI OF NY</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Conrad</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Kurumi</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Valter</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Market | Kokyutosu</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>BOBO</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The ProfessorX</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>770</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+210</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>KataChi</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Dmtr</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Scarlet</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Torune | Anbu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>San Pate Té</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>HASHIRAMA</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>BlacKaguya Ô</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Kiroi Senko</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>2988</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+384</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>BEBO</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>720</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>S3YL3</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>5188</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1816</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>YinRaku ™</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Ninja II</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>BlacKObito O</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>FEARLESS</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>™$£iko™°</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>2705</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+721</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>zDexTerx</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Archaic</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>11910</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+5168</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Nixervo</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>9430</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+4932</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Abyssteroth</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>12090</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+5172</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Floid</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Kojima</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>13033</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+4782</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>SharinganKniGhT</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ryujin 2ND</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>ANBU | HERO NICO 15</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UJKU SHIJAKUT </t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>RS | Oboy Max</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10645</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+4956</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>a_t_h_a_l_i_a</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>2780</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+310</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>SB | PapiiChan</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>6626</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+2504</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Envy</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>2242</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1479</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>RS | Oboy Lite</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10724</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+5061</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Haise</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>9685</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+3883</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Andres R</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-15 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3223.xlsx
+++ b/clan_3223.xlsx
@@ -37,6 +37,7 @@
     <sheet name="2026-08-11" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="2026-08-12" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="2026-08-14" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="2026-08-15" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21408,6 +21409,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sigma Brothers (3223)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-15 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>MAHORAGA</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>WoKy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>1208</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+1080</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>H U N T E R</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>SB ELISEUS</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>INFERNO</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>7813</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+1320</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Hydra anbu™</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Kyara Senju™</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>2335</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+1230</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Toka Senju™</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>GOJU</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>The prince JI OF NY</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Conrad</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Kurumi</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Valter</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Market | Kokyutosu</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>BOBO</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The ProfessorX</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>770</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>KataChi</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Dmtr</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Scarlet</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Torune | Anbu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>2880</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1620</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>San Pate Té</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>HASHIRAMA</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>310</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>BlacKaguya Ô</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Kiroi Senko</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>3288</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>BEBO</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1070</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>S3YL3</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>6210</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1022</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>YinRaku ™</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Ninja II</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>BlacKObito O</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>FEARLESS</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>™$£iko™°</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>3045</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+340</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>zDexTerx</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>960</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+960</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Archaic</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>14790</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+2820</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Nixervo</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>12310</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+2820</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Abyssteroth</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>14970</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+2820</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Floid</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Kojima</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>15859</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+2766</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>SharinganKniGhT</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ryujin 2ND</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>ANBU | HERO NICO 15</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UJKU SHIJAKUT </t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>RS | Oboy Max</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>12559</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+1854</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>a_t_h_a_l_i_a</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>5690</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+2660</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>SB | PapiiChan</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>7226</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Envy</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>2242</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>RS | Oboy Lite</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>13442</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+2658</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Haise</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>9985</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Andres R</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3223.xlsx
+++ b/clan_3223.xlsx
@@ -22298,7 +22298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-16 13:01:00</t>
+          <t>Timestamp: 2026-08-16 13:31:00</t>
         </is>
       </c>
     </row>
@@ -22881,11 +22881,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>22190</v>
+        <v>22358</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+7280</t>
+          <t>+7448</t>
         </is>
       </c>
     </row>
@@ -22896,11 +22896,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>19718</v>
+        <v>19886</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+7288</t>
+          <t>+7456</t>
         </is>
       </c>
     </row>
@@ -22911,11 +22911,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>22362</v>
+        <v>22530</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+7272</t>
+          <t>+7440</t>
         </is>
       </c>
     </row>
@@ -22941,11 +22941,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>22809</v>
+        <v>22977</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+6830</t>
+          <t>+6998</t>
         </is>
       </c>
     </row>
@@ -23031,11 +23031,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>19493</v>
+        <v>19661</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+6814</t>
+          <t>+6982</t>
         </is>
       </c>
     </row>
@@ -23091,11 +23091,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>20664</v>
+        <v>20832</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+7102</t>
+          <t>+7270</t>
         </is>
       </c>
     </row>
@@ -23106,11 +23106,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>13989</v>
+        <v>14157</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+4004</t>
+          <t>+4172</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-22 13:01:03
</commit_message>
<xml_diff>
--- a/clan_3223.xlsx
+++ b/clan_3223.xlsx
@@ -44,6 +44,7 @@
     <sheet name="2026-08-19" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="2026-08-20" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="2026-08-21" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="2026-08-22" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27478,6 +27479,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sigma Brothers (3223)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-22 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>MAHORAGA</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>WoKy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>7413</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>H U N T E R</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>SB ELISEUS</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>INFERNO</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>16808</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Kyara Senju™</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>16291</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+1700</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Toka Senju™</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>GOJU</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>The prince JI OF NY</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Conrad</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Kurumi</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Market | Kokyutosu</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>BOBO</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>The ProfessorX</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>10804</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>KataChi</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Dmtr</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+13</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Scarlet</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Torune | Anbu</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>17831</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1260</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>San Pate Té</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>N O G A R D</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>1091</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>HASHIRAMA</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>563</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>BlacKaguya Ô</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Kiroi Senko</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>3947</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>BEBO</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>4048</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>S3YL3</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>16651</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+920</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>YinRaku ™</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Suhaib</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>BlacKObito O</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>FEARLESS</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>™$£iko™°</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>4758</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>zDexTerx</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>17624</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+1800</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Archaic</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>40006</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1801</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Nixervo</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>37542</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+1801</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Abyssteroth</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>40346</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+1801</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Floid</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Kojima</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>44323</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+2820</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>SharinganKniGhT</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>BlacKenzie O</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ryujin 2ND</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UJKU SHIJAKUT </t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>BlacKEucresia Ó</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>912</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+612</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>RS | Oboy Max</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>37375</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+1617</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>a_t_h_a_l_i_a</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>28625</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+1841</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>SB | PapiiChan</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>9582</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Envy</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>2242</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>RS | Oboy Lite</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>36027</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Razor Sunkaze</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>1374</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+1082</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Haise</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>26627</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+1830</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Andres R</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-29 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3223.xlsx
+++ b/clan_3223.xlsx
@@ -34527,7 +34527,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-29 13:01:00</t>
+          <t>Timestamp: 2026-08-29 13:31:00</t>
         </is>
       </c>
     </row>
@@ -34720,11 +34720,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>818</v>
+        <v>3569</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+798</t>
+          <t>+3549</t>
         </is>
       </c>
     </row>
@@ -34840,11 +34840,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>14328</v>
+        <v>14928</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1318</t>
+          <t>+1918</t>
         </is>
       </c>
     </row>
@@ -34900,11 +34900,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>5882</v>
+        <v>6482</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -35050,11 +35050,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>40605</v>
+        <v>40725</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+2784</t>
+          <t>+2904</t>
         </is>
       </c>
     </row>
@@ -35065,11 +35065,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>63596</v>
+        <v>63636</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+2950</t>
+          <t>+2990</t>
         </is>
       </c>
     </row>
@@ -35125,11 +35125,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>69092</v>
+        <v>69212</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+2912</t>
+          <t>+3032</t>
         </is>
       </c>
     </row>
@@ -35185,11 +35185,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>23541</v>
+        <v>23901</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+2871</t>
+          <t>+3231</t>
         </is>
       </c>
     </row>
@@ -35335,11 +35335,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>9360</v>
+        <v>9840</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+1110</t>
+          <t>+1590</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-02 13:31:02
</commit_message>
<xml_diff>
--- a/clan_3223.xlsx
+++ b/clan_3223.xlsx
@@ -38047,7 +38047,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-02 13:01:00</t>
+          <t>Timestamp: 2026-09-02 13:31:01</t>
         </is>
       </c>
     </row>
@@ -38210,11 +38210,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>-17179</t>
+          <t>-17165</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-13 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3223.xlsx
+++ b/clan_3223.xlsx
@@ -49410,7 +49410,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-13 13:01:00</t>
+          <t>Timestamp: 2026-09-13 13:31:00</t>
         </is>
       </c>
     </row>
@@ -49693,11 +49693,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>22706</v>
+        <v>22773</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+4262</t>
+          <t>+4329</t>
         </is>
       </c>
     </row>
@@ -50038,11 +50038,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>32846</v>
+        <v>32946</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+4624</t>
+          <t>+4724</t>
         </is>
       </c>
     </row>
@@ -50083,11 +50083,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>14509</v>
+        <v>14629</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+4267</t>
+          <t>+4387</t>
         </is>
       </c>
     </row>
@@ -50143,11 +50143,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>16893</v>
+        <v>17193</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+3825</t>
+          <t>+4125</t>
         </is>
       </c>
     </row>
@@ -50158,11 +50158,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>24714</v>
+        <v>25114</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+3581</t>
+          <t>+3981</t>
         </is>
       </c>
     </row>
@@ -50203,11 +50203,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>25847</v>
+        <v>25867</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+3577</t>
+          <t>+3597</t>
         </is>
       </c>
     </row>

</xml_diff>